<commit_message>
Session 26 Task 1: Thesis Builder rulings (public companies on Incumbents, off Landscape, raised blank in energy_companies with the note public company; Capital investors and dates only with a quoted span from a cited source), both workbooks rebuilt from their saved states with --resume (no new calls)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/thesis/grid-scale-battery-storage-software-for-merchant-operators.xlsx
+++ b/docs/thesis/grid-scale-battery-storage-software-for-merchant-operators.xlsx
@@ -1188,7 +1188,7 @@
               <color rgb="00808080"/>
               <sz val="10"/>
             </rPr>
-            <t>2026-09-28 11:38 UTC by warehouse/thesis/build.py, run 20260928T112703Z; 24 model calls (claude-sonnet-5), 25 web searches, USD 2.4002, 11.5 minutes. Numbers not found in a cited source are written as not confirmed.</t>
+            <t>2026-09-28 17:07 UTC by warehouse/thesis/build.py, run 20260928T170427Z; 24 model calls (claude-sonnet-5), 25 web searches, USD 2.4002, 2.8 minutes. Numbers not found in a cited source are written as not confirmed.</t>
           </r>
         </is>
       </c>
@@ -2488,7 +2488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J16"/>
+  <dimension ref="B1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2923,102 +2923,8 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Fluence Energy</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Bid-optimization software (Mosaic) and asset performance management (Nispera) alongside battery-storage hardware products.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>not disclosed</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>public, Nasdaq: FLNC</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Revenue of $2.3 billion for fiscal year 2025; annual recurring revenue guidance of approximately $145 million for FY2025</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>not disclosed</t>
-        </is>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>Mosaic-optimized assets outperformed the CAISO market average by 50% in summer 2025; Mosaic has over 10GW of assets under management.</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>S18, S57, S68, S70, S143, S144</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>100: 3 independent sources, latest 2025; stage confirmed and raised confirmed by a primary source</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Stem, Inc.</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Athena AI platform and PowerTrack suite for asset performance management of storage, solar and hybrid portfolios.</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>not disclosed</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>public, NYSE: STEM</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Hardware revenue of $68.6 million in 2025, 43.9% of total revenue, per 10-K; accumulated deficit of $1,488.7 million</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>not disclosed</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>Contracted storage assets under management fell to nearly 2 GWh in 2025 after growing just 100MWh (5.5GWh to 5.6GWh) in 2024; shares traded 95.29% below their $10.00 IPO price.</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>S28, S35, S102</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>100: 3 independent sources, latest 2025; stage confirmed and raised confirmed by a primary source</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="345" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
+    <row r="14" ht="285" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3037,7 +2943,7 @@
               <color rgb="00808080"/>
               <sz val="10"/>
             </rPr>
-            <t>S91 Tyba raises $13.9M Series A to improve the profitability of ; S92 Tyba: Funding, Team &amp; Investors | Startup Intros; S93 Tyba raises $13.9M Series A to improve the profitability of ; S95 Tyba - 2026 Company Profile, Team, Funding &amp; Competitors - T; S97 Tyba raises $13.9M Series A to improve the profitability of ; S98 Tyba Raises $13.9 Million in Series A; S19 Habitat Energy - Crunchbase Company Profile &amp; Funding; S20 Canadian Solar invests in battery storage software company H; S22 Habitat Energy 2026 Company Profile: Valuation, Funding &amp; In; S23 Habitat Energy launches US Battery storage optimization plat; S25 What we do - Habitat Energy; S71 Danske Commodities and Habitat Energy win UK battery optimis; S73 Energy management startup GridBeyond funding round raises $1; S75 AI-driven optimiser GridBeyond raises €52 million from inves; S78 Powering progress: GridBeyond’s 2025 journey | GridBeyond; S81 GridBeyond - 2026 Company Profile, Team, Funding, Competitor; S37 Gridmatic Portfolio Investments, Gridmatic Funds, Gridmatic ; S39 Gridmatic US$50 million fund to manage battery storage proje; S90 Gridmatic Surpasses 1GWh of Energy Storage Under Management ; S111 Gridmatic - 2026 Company Profile, Team &amp; Competitors - Tracx; S89 Amperon | Demand Forecasts for the Energy Transition; S115 Amperon secures $20M series B, plans to expand platform - In; S119 How Much Did Amperon Raise? Funding &amp; Key Investors | Clay; S120 Amperon - 2026 Company Profile, Team, Funding &amp; Competitors ; S46 Schneider Electric set to acquire AutoGrid – pv magazine Int; S48 Schneider Electric to acquire AutoGrid, developer of AI for ; S49 Schneider Electric Acquires AutoGrid for an Undisclosed Amou; S51 Climate-AI Pioneer AutoGrid to Be Acquired by Schneider Elec; S52 Schneider Electric to buy out AutoGrid, combining AI optimiz; S108 Uplight to Acquire AutoGrid, Expanding Clean Energy Offering; S133 FlexGen Power Raises $100 Million in Series C Funding - Merc; S134 FlexGen's $100M Series C is the latest sign of the Southeast; S136 FlexGen Announces $100 Million Series C to Power Continued G; S137 Vitol invests in energy storage solutions provider FlexGen -; S140 FlexGen Announces $100 Million Series C to Power Continued G; S18 Fluence Energy FY2025 Annual Results: Revenue Down 16% to $2; S57 US battery energy storage operators and optimizers - and how; S68 Beating the Benchmark: Evolving Energy Storage Bidding in th; S70 Fluence Energy, Inc. - Form 10-K - FY2025; S143 Fluence Energy, Inc. - Form 8-K - FY2025; S144 Fluence Energy, Inc. - Form 8-K - FY2025; S28 Stem revenue down 69% in 2024 amid strategic shift away from; S35 Stem shifts to software-led model after restructuring | STEM; S102 STEM, INC. - Form 10-K - FY2024</t>
+            <t>S91 Tyba raises $13.9M Series A to improve the profitability of ; S92 Tyba: Funding, Team &amp; Investors | Startup Intros; S93 Tyba raises $13.9M Series A to improve the profitability of ; S95 Tyba - 2026 Company Profile, Team, Funding &amp; Competitors - T; S97 Tyba raises $13.9M Series A to improve the profitability of ; S98 Tyba Raises $13.9 Million in Series A; S19 Habitat Energy - Crunchbase Company Profile &amp; Funding; S20 Canadian Solar invests in battery storage software company H; S22 Habitat Energy 2026 Company Profile: Valuation, Funding &amp; In; S23 Habitat Energy launches US Battery storage optimization plat; S25 What we do - Habitat Energy; S71 Danske Commodities and Habitat Energy win UK battery optimis; S73 Energy management startup GridBeyond funding round raises $1; S75 AI-driven optimiser GridBeyond raises €52 million from inves; S78 Powering progress: GridBeyond’s 2025 journey | GridBeyond; S81 GridBeyond - 2026 Company Profile, Team, Funding, Competitor; S37 Gridmatic Portfolio Investments, Gridmatic Funds, Gridmatic ; S39 Gridmatic US$50 million fund to manage battery storage proje; S90 Gridmatic Surpasses 1GWh of Energy Storage Under Management ; S111 Gridmatic - 2026 Company Profile, Team &amp; Competitors - Tracx; S89 Amperon | Demand Forecasts for the Energy Transition; S115 Amperon secures $20M series B, plans to expand platform - In; S119 How Much Did Amperon Raise? Funding &amp; Key Investors | Clay; S120 Amperon - 2026 Company Profile, Team, Funding &amp; Competitors ; S46 Schneider Electric set to acquire AutoGrid – pv magazine Int; S48 Schneider Electric to acquire AutoGrid, developer of AI for ; S49 Schneider Electric Acquires AutoGrid for an Undisclosed Amou; S51 Climate-AI Pioneer AutoGrid to Be Acquired by Schneider Elec; S52 Schneider Electric to buy out AutoGrid, combining AI optimiz; S108 Uplight to Acquire AutoGrid, Expanding Clean Energy Offering; S133 FlexGen Power Raises $100 Million in Series C Funding - Merc; S134 FlexGen's $100M Series C is the latest sign of the Southeast; S136 FlexGen Announces $100 Million Series C to Power Continued G; S137 Vitol invests in energy storage solutions provider FlexGen -; S140 FlexGen Announces $100 Million Series C to Power Continued G</t>
           </r>
         </is>
       </c>
@@ -3045,7 +2951,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B14:I14"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3182,7 +3088,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Schneider Electric (buyer)</t>
+          <t>Schneider Electric</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -3219,7 +3125,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Vitol (anchor), existing investors</t>
+          <t>Vitol</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -3229,11 +3135,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>2023-10-03</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="inlineStr"/>
       <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Amperon</t>
@@ -3256,7 +3158,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Energize Capital (lead), D.E. Shaw group, Veriten, HSBC Asset Management</t>
+          <t>Energize Capital; Veriten; HSBC Asset Management</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -3266,11 +3168,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>2023-11-15</t>
-        </is>
-      </c>
+      <c r="B10" s="7" t="inlineStr"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Gridmatic</t>
@@ -3293,7 +3191,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>not named individually in release</t>
+          <t>not disclosed</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -3303,11 +3201,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
+      <c r="B11" s="6" t="inlineStr"/>
       <c r="C11" s="6" t="inlineStr">
         <is>
           <t>GridBeyond</t>
@@ -3330,7 +3224,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Energy Impact Partners, Yokogawa Electric, ABB, and others</t>
+          <t>Energy Impact Partners; ABB</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -3367,7 +3261,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Energize Capital (lead), Pear VC, Mobilize Climate Capital, Borusan Ventures; follow-on Powerhouse, Wireframe, Virta, Lorimer</t>
+          <t>Pear VC; Mobilize Climate Capital; Borusan Ventures; Wireframe</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -3377,11 +3271,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>2025-03-12</t>
-        </is>
-      </c>
+      <c r="B13" s="6" t="inlineStr"/>
       <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Amperon</t>
@@ -3402,11 +3292,7 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>National Grid Partners</t>
-        </is>
-      </c>
+      <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr">
         <is>
           <t>S119</t>
@@ -3414,11 +3300,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="B14" s="7" t="inlineStr"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
           <t>GridBeyond</t>
@@ -3441,7 +3323,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Samsung Ventures, ABB, Constellation, Act Venture Capital</t>
+          <t>Samsung Ventures; ABB; Constellation; Act Venture Capital</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -5507,7 +5389,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>'Scope'!B6; 'Scope'!B11:C11; 'Scope'!B16; 'Landscape'!B14:J14; 'Landscape'!B16</t>
+          <t>'Scope'!B6; 'Scope'!B11:C11; 'Scope'!B16</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5417,7 @@
       <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B8:J8; 'Landscape'!B16</t>
+          <t>'Landscape'!B8:J8; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5449,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B8:J8; 'Landscape'!B16</t>
+          <t>'Landscape'!B8:J8; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5509,7 @@
       <c r="F27" s="7" t="inlineStr"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>'Scope'!B6; 'Landscape'!B8:J8; 'Landscape'!B16; 'Risks'!B27</t>
+          <t>'Scope'!B6; 'Landscape'!B8:J8; 'Landscape'!B14; 'Risks'!B27</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5541,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B8:J8; 'Landscape'!B16</t>
+          <t>'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B8:J8; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5605,7 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B6; 'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B8:J8; 'Landscape'!B16</t>
+          <t>'Scope'!B6; 'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B8:J8; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -5811,7 +5693,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B15:J15; 'Landscape'!B16; 'Incumbents'!B14:H14; 'Incumbents'!B16; 'Risks'!B37</t>
+          <t>'Incumbents'!B14:H14; 'Incumbents'!B16; 'Risks'!B37</t>
         </is>
       </c>
     </row>
@@ -6027,7 +5909,7 @@
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>'Fundamentals'!B22:F22; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B15:J15; 'Landscape'!B16; 'Incumbents'!B11:H11; 'Incumbents'!B12:H12; 'Incumbents'!B13:H13; 'Incumbents'!B16; 'Risks'!B37</t>
+          <t>'Fundamentals'!B22:F22; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Incumbents'!B11:H11; 'Incumbents'!B12:H12; 'Incumbents'!B13:H13; 'Incumbents'!B16; 'Risks'!B37</t>
         </is>
       </c>
     </row>
@@ -6083,7 +5965,7 @@
       <c r="F42" s="6" t="inlineStr"/>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>'Fundamentals'!B24:F24; 'Fundamentals'!B27; 'Landscape'!B10:J10; 'Landscape'!B16; 'Capital'!B10:H10; 'Capital'!B15; 'Risks'!B27</t>
+          <t>'Fundamentals'!B24:F24; 'Fundamentals'!B27; 'Landscape'!B10:J10; 'Landscape'!B14; 'Capital'!B10:H10; 'Capital'!B15; 'Risks'!B27</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6029,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B12:C12; 'Scope'!B16; 'Fundamentals'!B24:F24; 'Fundamentals'!B27; 'Landscape'!B10:J10; 'Landscape'!B16; 'Capital'!B10:H10; 'Capital'!B15; 'Risks'!B12</t>
+          <t>'Scope'!B12:C12; 'Scope'!B16; 'Fundamentals'!B24:F24; 'Fundamentals'!B27; 'Landscape'!B10:J10; 'Landscape'!B14; 'Capital'!B10:H10; 'Capital'!B15; 'Risks'!B12</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6245,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16; 'Capital'!B7:H7; 'Capital'!B15</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14; 'Capital'!B7:H7; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -6427,7 +6309,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -6459,7 +6341,7 @@
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16; 'Capital'!B7:H7; 'Capital'!B15; 'Incumbents'!B15:H15; 'Incumbents'!B16; 'Risks'!B17</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14; 'Capital'!B7:H7; 'Capital'!B15; 'Incumbents'!B15:H15; 'Incumbents'!B16; 'Risks'!B17</t>
         </is>
       </c>
     </row>
@@ -6523,7 +6405,7 @@
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -6555,7 +6437,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -6715,7 +6597,7 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B6; 'Scope'!B13:C13; 'Scope'!B16; 'Fundamentals'!B21:F21; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B14:J14; 'Landscape'!B16; 'Incumbents'!B10:H10; 'Incumbents'!B16</t>
+          <t>'Scope'!B6; 'Scope'!B13:C13; 'Scope'!B16; 'Fundamentals'!B21:F21; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Incumbents'!B10:H10; 'Incumbents'!B16</t>
         </is>
       </c>
     </row>
@@ -7063,7 +6945,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B14:J14; 'Landscape'!B16</t>
+          <t>searched, not cited in a cell</t>
         </is>
       </c>
     </row>
@@ -7123,7 +7005,7 @@
       <c r="F75" s="7" t="inlineStr"/>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>'Scope'!B11:C11; 'Scope'!B16; 'Landscape'!B14:J14; 'Landscape'!B16</t>
+          <t>'Scope'!B11:C11; 'Scope'!B16</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7037,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B8:J8; 'Landscape'!B16</t>
+          <t>'Landscape'!B8:J8; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7097,7 @@
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B9:J9; 'Landscape'!B16; 'Capital'!B14:H14; 'Capital'!B15</t>
+          <t>'Landscape'!B9:J9; 'Landscape'!B14; 'Capital'!B14:H14; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -7279,7 +7161,7 @@
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B13:C13; 'Scope'!B16; 'Fundamentals'!B23:F23; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B9:J9; 'Landscape'!B16; 'Capital'!B11:H11; 'Capital'!B15</t>
+          <t>'Scope'!B13:C13; 'Scope'!B16; 'Fundamentals'!B23:F23; 'Fundamentals'!B27; 'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B9:J9; 'Landscape'!B14; 'Capital'!B11:H11; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -7375,7 +7257,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B9:J9; 'Landscape'!B16</t>
+          <t>'Landscape'!B9:J9; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7345,7 @@
       </c>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B9:J9; 'Landscape'!B16</t>
+          <t>'Landscape'!B9:J9; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7699,7 +7581,7 @@
       <c r="F94" s="6" t="inlineStr"/>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B11:J11; 'Landscape'!B16</t>
+          <t>'Landscape'!B11:J11; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7609,7 @@
       <c r="F95" s="7" t="inlineStr"/>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B10:J10; 'Landscape'!B16; 'Risks'!B7</t>
+          <t>'Trends'!B129:C129; 'Trends'!B130:C130; 'Trends'!B131:C131; 'Trends'!B132:C132; 'Trends'!B133; 'Landscape'!B10:J10; 'Landscape'!B14; 'Risks'!B7</t>
         </is>
       </c>
     </row>
@@ -7759,7 +7641,7 @@
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>'Fundamentals'!B26:F26; 'Fundamentals'!B27; 'Landscape'!B7:J7; 'Landscape'!B16; 'Capital'!B12:H12; 'Capital'!B15; 'Risks'!B27</t>
+          <t>'Fundamentals'!B26:F26; 'Fundamentals'!B27; 'Landscape'!B7:J7; 'Landscape'!B14; 'Capital'!B12:H12; 'Capital'!B15; 'Risks'!B27</t>
         </is>
       </c>
     </row>
@@ -7791,7 +7673,7 @@
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B7:J7; 'Landscape'!B16</t>
+          <t>'Landscape'!B7:J7; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7705,7 @@
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B7:J7; 'Landscape'!B16; 'Capital'!B12:H12; 'Capital'!B15</t>
+          <t>'Landscape'!B7:J7; 'Landscape'!B14; 'Capital'!B12:H12; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -7883,7 +7765,7 @@
       </c>
       <c r="G100" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B7:J7; 'Landscape'!B16</t>
+          <t>'Landscape'!B7:J7; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7943,7 +7825,7 @@
       </c>
       <c r="G102" s="6" t="inlineStr">
         <is>
-          <t>'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B7:J7; 'Landscape'!B16</t>
+          <t>'Scope'!B13:C13; 'Scope'!B16; 'Landscape'!B7:J7; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7857,7 @@
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B7:J7; 'Landscape'!B16</t>
+          <t>'Landscape'!B7:J7; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -8091,7 +7973,7 @@
       <c r="F107" s="7" t="inlineStr"/>
       <c r="G107" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B15:J15; 'Landscape'!B16</t>
+          <t>searched, not cited in a cell</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8161,7 @@
       </c>
       <c r="G113" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B12:J12; 'Landscape'!B16; 'Risks'!B17</t>
+          <t>'Landscape'!B12:J12; 'Landscape'!B14; 'Risks'!B17</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8253,7 @@
       </c>
       <c r="G116" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B10:J10; 'Landscape'!B16</t>
+          <t>'Landscape'!B10:J10; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -8491,7 +8373,7 @@
       </c>
       <c r="G120" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B11:J11; 'Landscape'!B16; 'Capital'!B9:H9; 'Capital'!B15</t>
+          <t>'Landscape'!B11:J11; 'Landscape'!B14; 'Capital'!B9:H9; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -8615,7 +8497,7 @@
       <c r="F124" s="6" t="inlineStr"/>
       <c r="G124" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B11:J11; 'Landscape'!B16; 'Capital'!B13:H13; 'Capital'!B15</t>
+          <t>'Landscape'!B11:J11; 'Landscape'!B14; 'Capital'!B13:H13; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8529,7 @@
       </c>
       <c r="G125" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B11:J11; 'Landscape'!B16</t>
+          <t>'Landscape'!B11:J11; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -9047,7 +8929,7 @@
       </c>
       <c r="G138" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B13:J13; 'Landscape'!B16</t>
+          <t>'Landscape'!B13:J13; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -9079,7 +8961,7 @@
       </c>
       <c r="G139" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B13:J13; 'Landscape'!B16</t>
+          <t>'Landscape'!B13:J13; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -9139,7 +9021,7 @@
       <c r="F141" s="7" t="inlineStr"/>
       <c r="G141" s="7" t="inlineStr">
         <is>
-          <t>'Landscape'!B13:J13; 'Landscape'!B16</t>
+          <t>'Landscape'!B13:J13; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -9171,7 +9053,7 @@
       </c>
       <c r="G142" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B13:J13; 'Landscape'!B16</t>
+          <t>'Landscape'!B13:J13; 'Landscape'!B14</t>
         </is>
       </c>
     </row>
@@ -9267,7 +9149,7 @@
       </c>
       <c r="G145" s="7" t="inlineStr">
         <is>
-          <t>'Fundamentals'!B25:F25; 'Fundamentals'!B27; 'Landscape'!B13:J13; 'Landscape'!B16; 'Capital'!B8:H8; 'Capital'!B15</t>
+          <t>'Fundamentals'!B25:F25; 'Fundamentals'!B27; 'Landscape'!B13:J13; 'Landscape'!B14; 'Capital'!B8:H8; 'Capital'!B15</t>
         </is>
       </c>
     </row>
@@ -9355,7 +9237,7 @@
       <c r="F148" s="6" t="inlineStr"/>
       <c r="G148" s="6" t="inlineStr">
         <is>
-          <t>'Landscape'!B14:J14; 'Landscape'!B16; 'Incumbents'!B8:H8; 'Incumbents'!B16</t>
+          <t>'Incumbents'!B8:H8; 'Incumbents'!B16</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9265,7 @@
       <c r="F149" s="7" t="inlineStr"/>
       <c r="G149" s="7" t="inlineStr">
         <is>
-          <t>'Fundamentals'!B20:F20; 'Fundamentals'!B27; 'Landscape'!B14:J14; 'Landscape'!B16; 'Incumbents'!B7:H7; 'Incumbents'!B16</t>
+          <t>'Fundamentals'!B20:F20; 'Fundamentals'!B27; 'Incumbents'!B7:H7; 'Incumbents'!B16</t>
         </is>
       </c>
     </row>

</xml_diff>